<commit_message>
Update estimate stamping to use hardcoded cells for project creation and BC sync
Replace dynamic `stampMappings` with hardcoded cell references in `server/projectRoutes.ts` and `server/autodesk/bcSync.ts` for estimate file generation.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 079d17c8-81ad-4ed1-8d19-38721a489fe7
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/umZYtFa
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-03.xlsx
+++ b/backups/proposal-log-2026-04-03.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="51">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -137,6 +137,33 @@
   </si>
   <si>
     <t>https://app.buildingconnected.com/opportunities/69bc538e7aaadb003896155f</t>
+  </si>
+  <si>
+    <t>26-0205</t>
+  </si>
+  <si>
+    <t>TRA General Office Complex</t>
+  </si>
+  <si>
+    <t>Dallas (DFW)</t>
+  </si>
+  <si>
+    <t>Office</t>
+  </si>
+  <si>
+    <t>2026-04-02</t>
+  </si>
+  <si>
+    <t>2026-04-23</t>
+  </si>
+  <si>
+    <t>Estimating</t>
+  </si>
+  <si>
+    <t>2026-08-03</t>
+  </si>
+  <si>
+    <t>2027-07-30</t>
   </si>
 </sst>
 </file>
@@ -535,7 +562,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -727,8 +754,52 @@
         <v>41</v>
       </c>
     </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F5" t="s">
+        <v>47</v>
+      </c>
+      <c r="G5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" t="s">
+        <v>48</v>
+      </c>
+      <c r="K5" t="s">
+        <v>49</v>
+      </c>
+      <c r="L5" t="s">
+        <v>50</v>
+      </c>
+      <c r="M5" t="s">
+        <v>17</v>
+      </c>
+      <c r="N5" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N4"/>
+  <autoFilter ref="A1:N5"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update folder naming to use only the airport code for clarity
Modify ProjectLogPage.tsx to extract the airport code from the region label for the folder preview display.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: f0ec7ae5-a290-402d-863b-f160d839a47d
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/j9R3Nur
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-03.xlsx
+++ b/backups/proposal-log-2026-04-03.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="95">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -164,6 +164,138 @@
   </si>
   <si>
     <t>2027-07-30</t>
+  </si>
+  <si>
+    <t>26-0214</t>
+  </si>
+  <si>
+    <t>UWMC ML TRU Pathology Lab</t>
+  </si>
+  <si>
+    <t>SEA</t>
+  </si>
+  <si>
+    <t>2026-04-03</t>
+  </si>
+  <si>
+    <t>Nick Jennings</t>
+  </si>
+  <si>
+    <t>Estimating</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69cfe3add7a6218079f9a6b3</t>
+  </si>
+  <si>
+    <t>26-0213</t>
+  </si>
+  <si>
+    <t>DFW</t>
+  </si>
+  <si>
+    <t>Christman Weeks</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69ce6ad9ffa00f5f6b96a4d9</t>
+  </si>
+  <si>
+    <t>26-0212</t>
+  </si>
+  <si>
+    <t>Adidas Tanger Deer Park</t>
+  </si>
+  <si>
+    <t>LGA</t>
+  </si>
+  <si>
+    <t>2026-04-08</t>
+  </si>
+  <si>
+    <t>Joseph Dinielli</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69cd0562786a720050b13b93</t>
+  </si>
+  <si>
+    <t>26-0211</t>
+  </si>
+  <si>
+    <t>Amazon SEA Legacy Space Refresh Medium GC Bid</t>
+  </si>
+  <si>
+    <t>2026-04-09</t>
+  </si>
+  <si>
+    <t>Merci Keathley</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69cc472c724d4f360623c300</t>
+  </si>
+  <si>
+    <t>26-0209</t>
+  </si>
+  <si>
+    <t>Flying Pickle Idaho Falls</t>
+  </si>
+  <si>
+    <t>GEG</t>
+  </si>
+  <si>
+    <t>Special Projects</t>
+  </si>
+  <si>
+    <t>2026-03-31</t>
+  </si>
+  <si>
+    <t>2026-04-13</t>
+  </si>
+  <si>
+    <t>Jake Marrujo</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69cc01834e68f2d35d122b59</t>
+  </si>
+  <si>
+    <t>26-0208</t>
+  </si>
+  <si>
+    <t>26-0207</t>
+  </si>
+  <si>
+    <t>Illumina Project SOL</t>
+  </si>
+  <si>
+    <t>SAN</t>
+  </si>
+  <si>
+    <t>2026-04-21</t>
+  </si>
+  <si>
+    <t>Vahid Balali</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69c6e1d59317e8e48f1c9603</t>
+  </si>
+  <si>
+    <t>26-0206</t>
+  </si>
+  <si>
+    <t>Inglewood Transit Connector RFQ</t>
+  </si>
+  <si>
+    <t>Retail</t>
+  </si>
+  <si>
+    <t>2026-03-25</t>
+  </si>
+  <si>
+    <t>2026-04-11</t>
+  </si>
+  <si>
+    <t>Nilda Puno</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69c42fb71e34da5627943f29</t>
   </si>
 </sst>
 </file>
@@ -562,7 +694,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -798,8 +930,360 @@
         <v>17</v>
       </c>
     </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" t="s">
+        <v>55</v>
+      </c>
+      <c r="I6" t="s">
+        <v>17</v>
+      </c>
+      <c r="J6" t="s">
+        <v>56</v>
+      </c>
+      <c r="K6" t="s">
+        <v>17</v>
+      </c>
+      <c r="L6" t="s">
+        <v>17</v>
+      </c>
+      <c r="M6" t="s">
+        <v>17</v>
+      </c>
+      <c r="N6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" t="s">
+        <v>59</v>
+      </c>
+      <c r="D7" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" t="s">
+        <v>46</v>
+      </c>
+      <c r="F7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G7" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7" t="s">
+        <v>60</v>
+      </c>
+      <c r="I7" t="s">
+        <v>17</v>
+      </c>
+      <c r="J7" t="s">
+        <v>56</v>
+      </c>
+      <c r="K7" t="s">
+        <v>17</v>
+      </c>
+      <c r="L7" t="s">
+        <v>17</v>
+      </c>
+      <c r="M7" t="s">
+        <v>17</v>
+      </c>
+      <c r="N7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" t="s">
+        <v>65</v>
+      </c>
+      <c r="G8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" t="s">
+        <v>66</v>
+      </c>
+      <c r="I8" t="s">
+        <v>17</v>
+      </c>
+      <c r="J8" t="s">
+        <v>56</v>
+      </c>
+      <c r="K8" t="s">
+        <v>17</v>
+      </c>
+      <c r="L8" t="s">
+        <v>17</v>
+      </c>
+      <c r="M8" t="s">
+        <v>17</v>
+      </c>
+      <c r="N8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>68</v>
+      </c>
+      <c r="B9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C9" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" t="s">
+        <v>70</v>
+      </c>
+      <c r="G9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" t="s">
+        <v>71</v>
+      </c>
+      <c r="I9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J9" t="s">
+        <v>56</v>
+      </c>
+      <c r="K9" t="s">
+        <v>17</v>
+      </c>
+      <c r="L9" t="s">
+        <v>17</v>
+      </c>
+      <c r="M9" t="s">
+        <v>17</v>
+      </c>
+      <c r="N9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" t="s">
+        <v>74</v>
+      </c>
+      <c r="C10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E10" t="s">
+        <v>77</v>
+      </c>
+      <c r="F10" t="s">
+        <v>78</v>
+      </c>
+      <c r="G10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" t="s">
+        <v>79</v>
+      </c>
+      <c r="I10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J10" t="s">
+        <v>56</v>
+      </c>
+      <c r="K10" t="s">
+        <v>17</v>
+      </c>
+      <c r="L10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N10" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>81</v>
+      </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" t="s">
+        <v>18</v>
+      </c>
+      <c r="F11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H11" t="s">
+        <v>20</v>
+      </c>
+      <c r="I11" t="s">
+        <v>17</v>
+      </c>
+      <c r="J11" t="s">
+        <v>56</v>
+      </c>
+      <c r="K11" t="s">
+        <v>17</v>
+      </c>
+      <c r="L11" t="s">
+        <v>17</v>
+      </c>
+      <c r="M11" t="s">
+        <v>17</v>
+      </c>
+      <c r="N11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>82</v>
+      </c>
+      <c r="B12" t="s">
+        <v>83</v>
+      </c>
+      <c r="C12" t="s">
+        <v>84</v>
+      </c>
+      <c r="D12" t="s">
+        <v>76</v>
+      </c>
+      <c r="E12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F12" t="s">
+        <v>85</v>
+      </c>
+      <c r="G12" t="s">
+        <v>17</v>
+      </c>
+      <c r="H12" t="s">
+        <v>86</v>
+      </c>
+      <c r="I12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J12" t="s">
+        <v>56</v>
+      </c>
+      <c r="K12" t="s">
+        <v>17</v>
+      </c>
+      <c r="L12" t="s">
+        <v>17</v>
+      </c>
+      <c r="M12" t="s">
+        <v>17</v>
+      </c>
+      <c r="N12" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>88</v>
+      </c>
+      <c r="B13" t="s">
+        <v>89</v>
+      </c>
+      <c r="C13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" t="s">
+        <v>90</v>
+      </c>
+      <c r="E13" t="s">
+        <v>91</v>
+      </c>
+      <c r="F13" t="s">
+        <v>92</v>
+      </c>
+      <c r="G13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H13" t="s">
+        <v>93</v>
+      </c>
+      <c r="I13" t="s">
+        <v>17</v>
+      </c>
+      <c r="J13" t="s">
+        <v>56</v>
+      </c>
+      <c r="K13" t="s">
+        <v>17</v>
+      </c>
+      <c r="L13" t="s">
+        <v>17</v>
+      </c>
+      <c r="M13" t="s">
+        <v>17</v>
+      </c>
+      <c r="N13" t="s">
+        <v>94</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N5"/>
+  <autoFilter ref="A1:N13"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>